<commit_message>
Fix Norwegian characters in test data categories
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/automation-agency/demo/RAPPORT_testdata_ror_as.xlsx
+++ b/automation-agency/demo/RAPPORT_testdata_ror_as.xlsx
@@ -496,7 +496,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generert: 13.03.2026 04:55</t>
+          <t>Generert: 13.03.2026 06:14</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid (161,958 NOK)</t>
+          <t>Rørleggerarbeid (161,958 NOK)</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Lonn assistent (61,487 NOK)</t>
+          <t>Lønn assistent (61,487 NOK)</t>
         </is>
       </c>
     </row>
@@ -655,10 +655,11 @@
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t># Økonomisk sammendrag for Testdata Rør AS
-Bedriften din har levert et solid resultat med 301 559 kroner i overskudd og en imponerende margin på 71 % – dette er godt over gjennomsnittet for bransjen. Rørleggerarbeid er den klare inntektsmotoren din og står for nesten 40 % av omsetningen. Den store forskjellen mellom beste måned (mars: 203 295 kr) og svakeste måned (januar: 15 058 kr) tyder på sesongsvingninger eller ujevn oppdragsflyt som det er verdt å følge med på. Lønnskostnader til assistent utgjør halvparten av utgiftene dine, noe som er normalt, men bør vurderes opp mot hvor mye inntekt assistenten bidrar til å generere.
+Du har levert et solid resultat med over 300 000 kroner i overskudd og en margin på 71 % – dette er svært sterkt for en håndverksbedrift. Rørleggerarbeid er din klare inntektsdriver og står for nesten 40 % av omsetningen. Det er verdt å merke seg den store forskjellen mellom beste og svakeste måned: mars ga over 13 ganger så godt resultat som januar.
 **Mine råd:**
-1. **Bygg en buffer:** Sett av 50 000–75 000 kr fra overskuddet til en driftskonto som dekker svake måneder som januar.
-2. **Utjevn sesongsvingningene:** Vurder å tilby serviceavtaler eller planlagt vedlikehold til faste kunder i rolige perioder – dette gir mer forutsigbar inntekt gjennom året.</t>
+1. Undersøk hva som gjorde mars så sterk – var det en stor jobb, sesongeffekt eller bedre kapasitetsutnyttelse? Bruk denne innsikten til å jevne ut svingningene.
+2. Lønnskostnader til assistent utgjør halvparten av utgiftene dine, så sørg for at timene utnyttes godt i roligere perioder, eventuelt gjennom vedlikeholdsavtaler eller planlagt arbeid.
+Du er godt posisjonert – nå handler det om å bygge forutsigbarhet.</t>
         </is>
       </c>
     </row>
@@ -772,7 +773,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -857,12 +858,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Lonn vikar</t>
+          <t>Lønn vikar</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lonn assistent</t>
+          <t>Lønn assistent</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -947,12 +948,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Sikkerhetsutsstyr</t>
+          <t>Sikkerhetsutstyr</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1007,7 +1008,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Avlopsdeler</t>
+          <t>Avløpsdeler</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1042,7 +1043,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1132,7 +1133,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1187,12 +1188,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lonn larling uke 3-4</t>
+          <t>Lønn lærling uke 3-4</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Lonn assistent</t>
+          <t>Lønn assistent</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1247,12 +1248,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Sikkerhetsutsstyr</t>
+          <t>Sikkerhetsutstyr</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1277,12 +1278,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Lonn larlingsassistent uke 1-2</t>
+          <t>Lønn lærlingassistent uke 1-2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Lonn assistent</t>
+          <t>Lønn assistent</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -1307,7 +1308,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Avlopsdeler</t>
+          <t>Avløpsdeler</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1337,12 +1338,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Utskifting av vannror kjokken</t>
+          <t>Utskifting av vannrør kjøkken</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1367,7 +1368,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Arsavtale vedlikehold</t>
+          <t>Årsavtale vedlikehold</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1432,7 +1433,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1492,7 +1493,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Lonn assistent</t>
+          <t>Lønn assistent</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1517,12 +1518,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nytt boreverktoy</t>
+          <t>Nytt boreverktøy</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1552,7 +1553,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1577,12 +1578,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Sikkerhetsutsstyr</t>
+          <t>Sikkerhetsutstyr</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1607,7 +1608,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Akutt rorbrudd natt</t>
+          <t>Akutt rørbrudd natt</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1637,12 +1638,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Lonn larlingsassistent uke 1-2</t>
+          <t>Lønn lærlingassistent uke 1-2</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Lonn assistent</t>
+          <t>Lønn assistent</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1732,7 +1733,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1757,7 +1758,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Akutt rorbrudd natt</t>
+          <t>Akutt rørbrudd natt</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1787,12 +1788,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Utskifting av vannror kjokken</t>
+          <t>Utskifting av vannrør kjøkken</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1847,12 +1848,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Nytt boreverktoy</t>
+          <t>Nytt boreverktøy</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -1882,7 +1883,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1907,12 +1908,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Sikkerhetsutsstyr</t>
+          <t>Sikkerhetsutstyr</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -1937,12 +1938,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Nytt boreverktoy</t>
+          <t>Nytt boreverktøy</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2032,7 +2033,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2062,7 +2063,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -2177,7 +2178,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Hasteoppdrag oversvommet kjeller</t>
+          <t>Hasteoppdrag oversvømt kjeller</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2237,7 +2238,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Arsavtale vedlikehold</t>
+          <t>Årsavtale vedlikehold</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2267,7 +2268,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Hasteoppdrag oversvommet kjeller</t>
+          <t>Hasteoppdrag oversvømt kjeller</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2297,7 +2298,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Arsservice varmeanlegg</t>
+          <t>Årsservice varmeanlegg</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2392,7 +2393,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2417,12 +2418,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Utskifting av vannror kjokken</t>
+          <t>Utskifting av vannrør kjøkken</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="F58" t="n">
@@ -2447,7 +2448,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Avlopsdeler</t>
+          <t>Avløpsdeler</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2561,7 +2562,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rorleggerarbeid</t>
+          <t>Rørleggerarbeid</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2673,7 +2674,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Verktoy</t>
+          <t>Verktøy</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -2705,7 +2706,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Lonn assistent</t>
+          <t>Lønn assistent</t>
         </is>
       </c>
       <c r="B11" t="n">

</xml_diff>